<commit_message>
Deploying to gh-pages from @ NIH-NCPI/ncpi-fhir-ig-2@c40062eec4c5ae05193f8fc349c7faabeb998778 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-adaptor-trimmed-cs.xlsx
+++ b/CodeSystem-adaptor-trimmed-cs.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-03T18:37:31+00:00</t>
+    <t>2025-12-03T22:26:51+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -72,7 +72,7 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>NCPI FHIR Working Group (http://example.org/example-publisher, ncpi-fhir-ig@googlegroups.com)</t>
+    <t>NCPI FHIR Working Group (https://www.ncpi-acc.org/about/working-groups, ncpi-fhir-ig@googlegroups.com)</t>
   </si>
   <si>
     <t>Jurisdiction</t>

</xml_diff>